<commit_message>
Day14 updates from class to github
</commit_message>
<xml_diff>
--- a/Language study.xlsx
+++ b/Language study.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\MBCA\Web\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCCEBB3F-8C3C-4162-9AA8-CDCAF5255AD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41FD609B-3378-4F78-9829-2C67DCA4C2B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{F2669019-19BE-4478-819B-56A03FBB98C4}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
   <si>
     <t xml:space="preserve">HTML </t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -120,6 +120,13 @@
   </si>
   <si>
     <t>&lt;div style="width:50%;"&gt;</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>대상객체.addEventListener(이벤트종류, 실행할함수);</t>
+  </si>
+  <si>
+    <t>message</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -178,7 +185,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -188,10 +195,7 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -508,7 +512,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D142731-8416-44C7-9CE6-C8C646A05D6B}">
-  <dimension ref="B1:L7"/>
+  <dimension ref="B1:L9"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="4" max="4" width="23.375" customWidth="1"/>
@@ -586,14 +590,14 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="2:12" s="3" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="3" t="s">
+    <row r="6" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B6" t="s">
         <v>21</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" t="s">
         <v>22</v>
       </c>
-      <c r="E6" s="4"/>
+      <c r="E6" s="3"/>
     </row>
     <row r="7" spans="2:12" ht="49.5" x14ac:dyDescent="0.3">
       <c r="B7" t="s">
@@ -601,6 +605,14 @@
       </c>
       <c r="E7" s="1" t="s">
         <v>16</v>
+      </c>
+    </row>
+    <row r="9" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="I9" t="s">
+        <v>24</v>
+      </c>
+      <c r="L9" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>